<commit_message>
update midtermreport and gantt chart
</commit_message>
<xml_diff>
--- a/DocumentsAndReports/updated_ghant_chart.xlsx
+++ b/DocumentsAndReports/updated_ghant_chart.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyawhein/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyawhein/cryto-streaming-pipeline/DocumentsAndReports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD344846-161A-FF4E-9D7D-D6D6EB26E5C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C166180-A6DF-2244-BF47-09DBF22D9242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16180" xr2:uid="{E5F47D3B-C3C5-4053-9D42-87F8D5301C97}"/>
   </bookViews>
@@ -1132,7 +1132,7 @@
         <v>25</v>
       </c>
       <c r="I8" s="22">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="J8" s="8"/>
       <c r="K8" s="8"/>
@@ -1177,7 +1177,7 @@
         <v>25</v>
       </c>
       <c r="I9" s="22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="8"/>
       <c r="K9" s="8"/>
@@ -1219,10 +1219,10 @@
         <v>4</v>
       </c>
       <c r="H10" s="21" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I10" s="22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" s="8"/>
       <c r="K10" s="8"/>

</xml_diff>